<commit_message>
updated code review comments
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramakrishna.tummala\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAF5EB70-1C71-4727-8EA4-08903D94487C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AE6EE51-E614-4733-93B8-301E66E27FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="117">
   <si>
     <t>Name</t>
   </si>
@@ -103,9 +103,6 @@
 HCAD NOHExtractor Automation process Bot completed the run successfully.&lt;br /&gt;&lt;br /&gt;
 Regards,&lt;br /&gt;
 RPA Automation</t>
-  </si>
-  <si>
-    <t>Failure: System Exception - HCAD NOHExtractor Automation</t>
   </si>
   <si>
     <t>Email_Details</t>
@@ -401,12 +398,42 @@
   <si>
     <t>ReadNOHEmailsFailed</t>
   </si>
+  <si>
+    <t>DestinationFolderPath</t>
+  </si>
+  <si>
+    <t>InProgress|Failed|Completed</t>
+  </si>
+  <si>
+    <t>EmailFolderInProgress</t>
+  </si>
+  <si>
+    <t>InProgress</t>
+  </si>
+  <si>
+    <t>Data Source=D-SQLREPORTS-02;Initial Catalog=Process_Dashboard;User ID=VendorDBO;Password=!V3nd0rDb02024Hc@D!;Encrypt=False</t>
+  </si>
+  <si>
+    <t>SqlConnectionString</t>
+  </si>
+  <si>
+    <t>Data Source={0};Initial Catalog={1};User ID={2};Password={3};Encrypt=False</t>
+  </si>
+  <si>
+    <t>Data Source=D-SQLREPORTS-02;Initial Catalog=Process_Dashboard;User ID={0};Password={1};Encrypt=False</t>
+  </si>
+  <si>
+    <t>StopProcessAfter</t>
+  </si>
+  <si>
+    <t>Failure: System Exception - HCAD SKED_Dispatcher Automation</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -451,6 +478,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -494,7 +528,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -527,6 +561,9 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -843,7 +880,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z937"/>
+  <dimension ref="A1:Z941"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34.81640625" bestFit="1" customWidth="1"/>
@@ -888,10 +925,10 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>6</v>
@@ -899,19 +936,19 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>69</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>70</v>
       </c>
       <c r="C4" s="5"/>
     </row>
@@ -920,7 +957,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>9</v>
@@ -931,7 +968,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>7</v>
@@ -939,404 +976,437 @@
     </row>
     <row r="7" spans="1:26" ht="14.5">
       <c r="A7" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>58</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>59</v>
       </c>
       <c r="C7" s="7"/>
     </row>
     <row r="8" spans="1:26" ht="14.5">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C8" s="7"/>
     </row>
     <row r="9" spans="1:26" ht="14.5">
       <c r="A9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C9" s="7"/>
     </row>
     <row r="10" spans="1:26" ht="14.5">
       <c r="A10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B10" s="16">
-        <v>100</v>
+        <v>65</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>33</v>
       </c>
       <c r="C10" s="7"/>
     </row>
     <row r="11" spans="1:26" ht="14.5">
       <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="16" t="s">
         <v>67</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>68</v>
       </c>
       <c r="C11" s="7"/>
     </row>
     <row r="12" spans="1:26" ht="14.5">
       <c r="A12" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.5">
       <c r="A13" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B13" s="14" t="s">
-        <v>83</v>
-      </c>
       <c r="C13" s="7"/>
     </row>
-    <row r="14" spans="1:26" ht="14.5">
+    <row r="14" spans="1:26" ht="29">
       <c r="A14" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="B14" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="C14" s="7"/>
+      <c r="C14" s="7" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="15" spans="1:26" ht="14.5">
       <c r="A15" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="B15" s="17" t="s">
         <v>90</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>89</v>
       </c>
       <c r="C15" s="7"/>
     </row>
     <row r="16" spans="1:26" ht="14.5">
       <c r="A16" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" s="17" t="s">
         <v>92</v>
-      </c>
-      <c r="B16" s="17" t="s">
-        <v>93</v>
       </c>
       <c r="C16" s="7"/>
     </row>
     <row r="17" spans="1:3" ht="101" customHeight="1">
       <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" s="17" t="s">
         <v>98</v>
-      </c>
-      <c r="B17" s="17" t="s">
-        <v>99</v>
       </c>
       <c r="C17" s="7"/>
     </row>
     <row r="18" spans="1:3" ht="29">
       <c r="A18" t="s">
+        <v>99</v>
+      </c>
+      <c r="B18" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="B18" s="17" t="s">
-        <v>101</v>
-      </c>
       <c r="C18" s="7"/>
     </row>
-    <row r="19" spans="1:3" ht="21">
-      <c r="A19" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="6"/>
-    </row>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A20" s="9" t="s">
-        <v>17</v>
+    <row r="19" spans="1:3" ht="14.5">
+      <c r="A19" t="s">
+        <v>107</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="14.5">
+      <c r="A20" t="s">
+        <v>109</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="6"/>
-    </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A21" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="6"/>
-    </row>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A22" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="C22" s="6"/>
-    </row>
-    <row r="23" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A23" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B23" s="18" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="14.5">
+      <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" t="s">
+        <v>113</v>
+      </c>
+      <c r="C21" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="14.5">
+      <c r="A22" t="s">
+        <v>115</v>
+      </c>
+      <c r="B22">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="21">
+      <c r="A23" s="8" t="s">
         <v>21</v>
       </c>
+      <c r="B23" s="14"/>
       <c r="C23" s="6"/>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" s="6"/>
+    </row>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A25" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="6"/>
+    </row>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A26" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="6"/>
+    </row>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A27" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="C27" s="6"/>
+    </row>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A28" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C28" s="6"/>
+    </row>
+    <row r="29" spans="1:3" ht="107.5" customHeight="1">
+      <c r="A29" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="B24" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="C24" s="6"/>
-    </row>
-    <row r="25" spans="1:3" ht="107.5" customHeight="1">
-      <c r="A25" s="9" t="s">
+      <c r="B29" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="B25" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" s="6"/>
-    </row>
-    <row r="26" spans="1:3" ht="21">
-      <c r="A26" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="14"/>
-      <c r="C26" s="6"/>
-    </row>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A27" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B27" s="2">
-        <v>3</v>
-      </c>
-      <c r="C27" s="6"/>
-    </row>
-    <row r="28" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A28" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C28" s="6"/>
-    </row>
-    <row r="29" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A29" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="C29" s="6"/>
     </row>
-    <row r="30" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A30" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>28</v>
-      </c>
+    <row r="30" spans="1:3" ht="21">
+      <c r="A30" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" s="14"/>
       <c r="C30" s="6"/>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="B31" s="2">
+        <v>3</v>
       </c>
       <c r="C31" s="6"/>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C32" s="6"/>
     </row>
     <row r="33" spans="1:3" ht="14.25" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="C33" s="6"/>
     </row>
     <row r="34" spans="1:3" ht="14.25" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C34" s="6"/>
     </row>
     <row r="35" spans="1:3" ht="14.25" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B35" s="2">
-        <v>2</v>
+        <v>28</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="C35" s="6"/>
     </row>
     <row r="36" spans="1:3" ht="14.25" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C36" s="6"/>
     </row>
     <row r="37" spans="1:3" ht="14.25" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C37" s="6"/>
     </row>
     <row r="38" spans="1:3" ht="14.25" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C38" s="6"/>
     </row>
     <row r="39" spans="1:3" ht="14.25" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>41</v>
+        <v>10</v>
+      </c>
+      <c r="B39" s="2">
+        <v>2</v>
       </c>
       <c r="C39" s="6"/>
     </row>
     <row r="40" spans="1:3" ht="14.25" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="C40" s="6"/>
     </row>
     <row r="41" spans="1:3" ht="14.25" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C41" s="6"/>
     </row>
     <row r="42" spans="1:3" ht="14.25" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C42" s="6"/>
     </row>
     <row r="43" spans="1:3" ht="14.25" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B43" s="2">
-        <v>2</v>
+        <v>39</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="C43" s="6"/>
     </row>
     <row r="44" spans="1:3" ht="14.25" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B44" s="2">
-        <v>2</v>
+        <v>41</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="C44" s="6"/>
     </row>
     <row r="45" spans="1:3" ht="14.25" customHeight="1">
       <c r="A45" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B45" s="3" t="b">
+        <v>43</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C45" s="6"/>
+    </row>
+    <row r="46" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C46" s="6"/>
+    </row>
+    <row r="47" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" s="2">
+        <v>2</v>
+      </c>
+      <c r="C47" s="6"/>
+    </row>
+    <row r="48" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B48" s="2">
+        <v>2</v>
+      </c>
+      <c r="C48" s="6"/>
+    </row>
+    <row r="49" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B49" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="C45" s="6"/>
-    </row>
-    <row r="46" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="47" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A47" s="10" t="s">
+      <c r="C49" s="6"/>
+    </row>
+    <row r="50" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="51" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A51" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="19" t="s">
+      <c r="B51" s="19" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A48" t="s">
+    <row r="52" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="B48" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A49" t="s">
+    </row>
+    <row r="53" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A53" t="s">
+        <v>102</v>
+      </c>
+      <c r="B53" s="16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A54" t="s">
+        <v>104</v>
+      </c>
+      <c r="B54" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="B49" s="16" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A50" t="s">
+    </row>
+    <row r="55" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A55" t="s">
+        <v>106</v>
+      </c>
+      <c r="B55" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="B50" s="16" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A51" t="s">
-        <v>107</v>
-      </c>
-      <c r="B51" s="16" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="53" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="54" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="57" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="59" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="62" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="63" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="64" spans="1:2" ht="14.25" customHeight="1"/>
+    </row>
+    <row r="56" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="57" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="58" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="59" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="60" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="61" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="62" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="63" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="64" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="65" ht="14.25" customHeight="1"/>
     <row r="66" ht="14.25" customHeight="1"/>
     <row r="67" ht="14.25" customHeight="1"/>
@@ -2210,6 +2280,10 @@
     <row r="935" ht="14.25" customHeight="1"/>
     <row r="936" ht="14.25" customHeight="1"/>
     <row r="937" ht="14.25" customHeight="1"/>
+    <row r="938" ht="14.25" customHeight="1"/>
+    <row r="939" ht="14.25" customHeight="1"/>
+    <row r="940" ht="14.25" customHeight="1"/>
+    <row r="941" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2236,98 +2310,98 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" t="s">
         <v>74</v>
-      </c>
-      <c r="B5" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B12" t="s">
         <v>84</v>
-      </c>
-      <c r="B12" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" t="s">
         <v>86</v>
-      </c>
-      <c r="B13" t="s">
-        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added insert datatable row
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramakrishna.tummala\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AE6EE51-E614-4733-93B8-301E66E27FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E1C11EB-6A94-4039-94D4-9D6A51DB9F06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="118">
   <si>
     <t>Name</t>
   </si>
@@ -427,6 +427,9 @@
   </si>
   <si>
     <t>Failure: System Exception - HCAD SKED_Dispatcher Automation</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1009,7 @@
         <v>65</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>33</v>
+        <v>117</v>
       </c>
       <c r="C10" s="7"/>
     </row>
@@ -1115,7 +1118,7 @@
         <v>115</v>
       </c>
       <c r="B22">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="21">

</xml_diff>